<commit_message>
Added new RDF data schemes and visual schemes for economy-table71-74, and fixed XLSX spreadsheets for economy-table72-73
</commit_message>
<xml_diff>
--- a/sources/table_normalization/xlsx/economy-table72.xlsx
+++ b/sources/table_normalization/xlsx/economy-table72.xlsx
@@ -106,9 +106,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="3">
-    <numFmt numFmtId="167" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0;[Red]\-&quot;$&quot;#,##0"/>
-    <numFmt numFmtId="169" formatCode="_-&quot;$&quot;* #,##0_-;\-&quot;$&quot;* #,##0_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0;[Red]\-&quot;$&quot;#,##0"/>
+    <numFmt numFmtId="166" formatCode="_-&quot;$&quot;* #,##0_-;\-&quot;$&quot;* #,##0_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -150,7 +150,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -172,6 +172,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -246,37 +252,33 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="168" fontId="2" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="2" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="168" fontId="2" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="2" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="5" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -768,15 +770,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="23.5">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="1"/>
@@ -800,7 +802,7 @@
       </c>
     </row>
     <row r="3" spans="1:7" ht="29">
-      <c r="A3" s="12" t="s">
+      <c r="A3" s="8" t="s">
         <v>7</v>
       </c>
       <c r="B3" s="1"/>
@@ -823,60 +825,60 @@
       <c r="A5" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="9" t="s">
+      <c r="B5" s="5" t="s">
         <v>9</v>
       </c>
       <c r="C5" s="1"/>
-      <c r="D5" s="9" t="s">
+      <c r="D5" s="5" t="s">
         <v>9</v>
       </c>
       <c r="E5" s="1"/>
-      <c r="F5" s="9" t="s">
+      <c r="F5" s="5" t="s">
         <v>10</v>
       </c>
       <c r="G5" s="1"/>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" s="1"/>
-      <c r="B6" s="9" t="s">
+      <c r="B6" s="5" t="s">
         <v>11</v>
       </c>
       <c r="C6" s="1"/>
-      <c r="D6" s="9" t="s">
+      <c r="D6" s="5" t="s">
         <v>11</v>
       </c>
       <c r="E6" s="1"/>
-      <c r="F6" s="9" t="s">
+      <c r="F6" s="5" t="s">
         <v>12</v>
       </c>
       <c r="G6" s="1"/>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" s="1"/>
-      <c r="B7" s="9" t="s">
+      <c r="B7" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C7" s="1"/>
-      <c r="D7" s="9" t="s">
+      <c r="D7" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E7" s="1"/>
-      <c r="F7" s="9" t="s">
+      <c r="F7" s="5" t="s">
         <v>14</v>
       </c>
       <c r="G7" s="1"/>
     </row>
     <row r="8" spans="1:7">
       <c r="A8" s="1"/>
-      <c r="B8" s="10">
+      <c r="B8" s="6">
         <v>10000</v>
       </c>
       <c r="C8" s="1"/>
-      <c r="D8" s="10">
+      <c r="D8" s="6">
         <v>10000</v>
       </c>
       <c r="E8" s="1"/>
-      <c r="F8" s="10">
+      <c r="F8" s="6">
         <v>15000</v>
       </c>
       <c r="G8" s="1"/>
@@ -892,11 +894,11 @@
     </row>
     <row r="10" spans="1:7">
       <c r="A10" s="1"/>
-      <c r="B10" s="11" t="s">
+      <c r="B10" s="7" t="s">
         <v>15</v>
       </c>
       <c r="C10" s="1"/>
-      <c r="D10" s="11" t="s">
+      <c r="D10" s="7" t="s">
         <v>15</v>
       </c>
       <c r="E10" s="1"/>
@@ -905,11 +907,11 @@
     </row>
     <row r="11" spans="1:7">
       <c r="A11" s="1"/>
-      <c r="B11" s="9" t="s">
+      <c r="B11" s="5" t="s">
         <v>11</v>
       </c>
       <c r="C11" s="1"/>
-      <c r="D11" s="9" t="s">
+      <c r="D11" s="5" t="s">
         <v>11</v>
       </c>
       <c r="E11" s="1"/>
@@ -918,11 +920,11 @@
     </row>
     <row r="12" spans="1:7">
       <c r="A12" s="1"/>
-      <c r="B12" s="9" t="s">
+      <c r="B12" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C12" s="1"/>
-      <c r="D12" s="9" t="s">
+      <c r="D12" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E12" s="1"/>
@@ -931,11 +933,11 @@
     </row>
     <row r="13" spans="1:7">
       <c r="A13" s="1"/>
-      <c r="B13" s="10">
+      <c r="B13" s="6">
         <v>8000</v>
       </c>
       <c r="C13" s="1"/>
-      <c r="D13" s="10">
+      <c r="D13" s="6">
         <v>8000</v>
       </c>
       <c r="E13" s="1"/>
@@ -964,14 +966,14 @@
       <c r="A16" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B16" s="9" t="s">
+      <c r="B16" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="C16" s="9" t="s">
+      <c r="C16" s="5" t="s">
         <v>17</v>
       </c>
       <c r="D16" s="1"/>
-      <c r="E16" s="9" t="s">
+      <c r="E16" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F16" s="1"/>
@@ -979,14 +981,14 @@
     </row>
     <row r="17" spans="1:7">
       <c r="A17" s="1"/>
-      <c r="B17" s="9" t="s">
+      <c r="B17" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C17" s="9" t="s">
+      <c r="C17" s="5" t="s">
         <v>18</v>
       </c>
       <c r="D17" s="1"/>
-      <c r="E17" s="9" t="s">
+      <c r="E17" s="5" t="s">
         <v>18</v>
       </c>
       <c r="F17" s="1"/>
@@ -994,14 +996,14 @@
     </row>
     <row r="18" spans="1:7">
       <c r="A18" s="1"/>
-      <c r="B18" s="9" t="s">
+      <c r="B18" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="C18" s="9" t="s">
+      <c r="C18" s="5" t="s">
         <v>19</v>
       </c>
       <c r="D18" s="1"/>
-      <c r="E18" s="9" t="s">
+      <c r="E18" s="5" t="s">
         <v>19</v>
       </c>
       <c r="F18" s="1"/>
@@ -1009,14 +1011,14 @@
     </row>
     <row r="19" spans="1:7">
       <c r="A19" s="1"/>
-      <c r="B19" s="10">
+      <c r="B19" s="6">
         <v>15000</v>
       </c>
-      <c r="C19" s="10">
+      <c r="C19" s="6">
         <v>10000</v>
       </c>
       <c r="D19" s="1"/>
-      <c r="E19" s="10">
+      <c r="E19" s="6">
         <v>10000</v>
       </c>
       <c r="F19" s="1"/>
@@ -1090,11 +1092,11 @@
         <v>20</v>
       </c>
       <c r="B27" s="1"/>
-      <c r="C27" s="4" t="s">
+      <c r="C27" s="5" t="s">
         <v>21</v>
       </c>
       <c r="D27" s="1"/>
-      <c r="E27" s="4" t="s">
+      <c r="E27" s="5" t="s">
         <v>21</v>
       </c>
       <c r="F27" s="1"/>
@@ -1103,11 +1105,11 @@
     <row r="28" spans="1:7">
       <c r="A28" s="1"/>
       <c r="B28" s="1"/>
-      <c r="C28" s="4" t="s">
+      <c r="C28" s="5" t="s">
         <v>11</v>
       </c>
       <c r="D28" s="1"/>
-      <c r="E28" s="4" t="s">
+      <c r="E28" s="5" t="s">
         <v>11</v>
       </c>
       <c r="F28" s="1"/>
@@ -1116,11 +1118,11 @@
     <row r="29" spans="1:7">
       <c r="A29" s="1"/>
       <c r="B29" s="1"/>
-      <c r="C29" s="4" t="s">
+      <c r="C29" s="5" t="s">
         <v>22</v>
       </c>
       <c r="D29" s="1"/>
-      <c r="E29" s="4" t="s">
+      <c r="E29" s="5" t="s">
         <v>22</v>
       </c>
       <c r="F29" s="1"/>
@@ -1129,11 +1131,11 @@
     <row r="30" spans="1:7">
       <c r="A30" s="1"/>
       <c r="B30" s="1"/>
-      <c r="C30" s="5">
+      <c r="C30" s="6">
         <v>12900</v>
       </c>
       <c r="D30" s="1"/>
-      <c r="E30" s="5">
+      <c r="E30" s="6">
         <v>12900</v>
       </c>
       <c r="F30" s="1"/>
@@ -1167,30 +1169,30 @@
       <c r="G33" s="1"/>
     </row>
     <row r="34" spans="1:7" ht="46.5">
-      <c r="A34" s="6" t="s">
+      <c r="A34" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="B34" s="7">
+      <c r="B34" s="4">
         <f t="shared" ref="B34:G34" si="0">SUM(B5:B33)</f>
         <v>33000</v>
       </c>
-      <c r="C34" s="7">
+      <c r="C34" s="4">
         <f t="shared" si="0"/>
         <v>22900</v>
       </c>
-      <c r="D34" s="7">
+      <c r="D34" s="4">
         <f t="shared" si="0"/>
         <v>18000</v>
       </c>
-      <c r="E34" s="7">
+      <c r="E34" s="4">
         <f t="shared" si="0"/>
         <v>22900</v>
       </c>
-      <c r="F34" s="7">
+      <c r="F34" s="4">
         <f t="shared" si="0"/>
         <v>15000</v>
       </c>
-      <c r="G34" s="7">
+      <c r="G34" s="4">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>

</xml_diff>